<commit_message>
feat: add M8 Test Execution skill files
</commit_message>
<xml_diff>
--- a/resources/template/tester/test_design/DefaultTestCaseTemplate.xlsx
+++ b/resources/template/tester/test_design/DefaultTestCaseTemplate.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -466,6 +466,8 @@
     <col width="24" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="32" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -547,6 +549,16 @@
       <c r="P1" t="inlineStr">
         <is>
           <t>用例状态</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>关联需求</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>所属项目</t>
         </is>
       </c>
     </row>

</xml_diff>